<commit_message>
Update Takataka Ids.xlsx with latest truck asset mappings for weekly dispatch.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Takataka Ids.xlsx
+++ b/Takataka Ids.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="7510"/>
+    <workbookView windowWidth="19200" windowHeight="8710"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>ReportName</t>
   </si>
@@ -35,37 +35,13 @@
     <t>itemId</t>
   </si>
   <si>
-    <t>FH-KCH146N</t>
-  </si>
-  <si>
     <t>TakaTaka - KCA074W</t>
-  </si>
-  <si>
-    <t>TakaTaka - KCK236X</t>
-  </si>
-  <si>
-    <t>TOYOTA DYNA-KCH227R</t>
   </si>
   <si>
     <t>HINO 300-KCW255E</t>
   </si>
   <si>
-    <t>BONGO MAZDA-KDB413K</t>
-  </si>
-  <si>
-    <t>HINO 500-KBZ179X</t>
-  </si>
-  <si>
-    <t>Taka Taka - KMEH040S</t>
-  </si>
-  <si>
     <t>TakaTaka - KBP335Q</t>
-  </si>
-  <si>
-    <t>HINO 500-KBZ178X</t>
-  </si>
-  <si>
-    <t>FUSO F1-KDK796G</t>
   </si>
   <si>
     <t>FUSO F1-KDK708G</t>
@@ -74,34 +50,19 @@
     <t>HINO 500-KCA836U</t>
   </si>
   <si>
-    <t>FUSO FN627-KDK794G</t>
-  </si>
-  <si>
     <t>CANTER-KDK022Y</t>
   </si>
   <si>
     <t>FH-KCA947V</t>
   </si>
   <si>
-    <t>CANTER-KDL106W</t>
-  </si>
-  <si>
-    <t>CANTER-KDM251W</t>
-  </si>
-  <si>
-    <t>FUSO F1-KDM085Y</t>
-  </si>
-  <si>
     <t>FUSO F1-KDM086Y</t>
-  </si>
-  <si>
-    <t>HINO 500-KBV226X</t>
   </si>
   <si>
     <t>FH-KCE699P</t>
   </si>
   <si>
-    <t>Canter-KBR235B</t>
+    <t>FUSO F1-KDK796G</t>
   </si>
 </sst>
 </file>
@@ -131,11 +92,10 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <u/>
@@ -282,12 +242,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -600,19 +566,19 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -621,7 +587,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -645,16 +611,16 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -663,93 +629,97 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -763,7 +733,7 @@
     <cellStyle name="Note" xfId="8" builtinId="10"/>
     <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
     <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
     <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
     <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
     <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
@@ -1096,7 +1066,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="24.2727272727273" customWidth="1"/>
@@ -1115,185 +1085,93 @@
       <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="3">
-        <v>19257066</v>
+      <c r="B2" s="4">
+        <v>19287792</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="3">
-        <v>19287792</v>
+      <c r="B3" s="4">
+        <v>20621455</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="3">
-        <v>19327513</v>
+      <c r="B4" s="4">
+        <v>23761333</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="3">
-        <v>19606459</v>
+      <c r="B5" s="4">
+        <v>26410109</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="3">
-        <v>20621455</v>
+      <c r="B6" s="4">
+        <v>26418733</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="3">
-        <v>22750817</v>
+      <c r="B7" s="4">
+        <v>26485232</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="3">
-        <v>23348505</v>
+      <c r="B8" s="4">
+        <v>26672025</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="3">
-        <v>23403505</v>
+      <c r="B9" s="4">
+        <v>27321125</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="3">
-        <v>23761333</v>
+      <c r="B10" s="4">
+        <v>27632811</v>
       </c>
     </row>
     <row r="11" spans="1:2">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="3">
-        <v>25838198</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2">
-      <c r="A12" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B12" s="3">
+      <c r="B11" s="4">
         <v>26405794</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
-      <c r="A13" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B13" s="3">
-        <v>26410109</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2">
-      <c r="A14" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B14" s="3">
-        <v>26418733</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2">
-      <c r="A15" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B15" s="3">
-        <v>26437421</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2">
-      <c r="A16" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B16" s="3">
-        <v>26485232</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2">
-      <c r="A17" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B17" s="3">
-        <v>26672025</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2">
-      <c r="A18" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B18" s="3">
-        <v>27026854</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2">
-      <c r="A19" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B19" s="3">
-        <v>27287873</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2">
-      <c r="A20" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B20" s="3">
-        <v>27321018</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2">
-      <c r="A21" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="B21" s="3">
-        <v>27321125</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2">
-      <c r="A22" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B22" s="3">
-        <v>27630984</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2">
-      <c r="A23" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B23" s="3">
-        <v>27632811</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2">
-      <c r="A24" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B24" s="3">
-        <v>27947252</v>
-      </c>
+    <row r="12" ht="15.5" spans="1:2">
+      <c r="A12" s="5"/>
+    </row>
+    <row r="13" ht="15.5" spans="1:2">
+      <c r="A13" s="5"/>
+    </row>
+    <row r="14" ht="15.5" spans="1:2">
+      <c r="A14" s="5"/>
+    </row>
+    <row r="15" ht="15.5" spans="1:2">
+      <c r="A15" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>